<commit_message>
Add Products section: per-campaign Y/N product toggles
Not every campaign runs every product, so the template now has a Products
section of Yes/No toggles. Blank = the brand's default set; No drops a product;
Yes adds one the brand supports (the after_midroll_bumper family maps to the
brand's specific bumper).

- models.py: PRODUCT_FAMILIES + SupportPlan.product_overrides.
- plan_loader: _apply_product_overrides after formats derive from the brand.
- gsheets: PRODUCT_TOGGLES + Plan-tab bool fields; Formats moved to Overrides.
- salesforce: Include_*__c Case fields (Yes/No) coerced to bool.
- workbook generator: Yes/No dropdowns on the 8 toggles (shared _Lists column).
- Plan.csv template + PLAN_TEMPLATE.md + salesforce-case-fields.csv updated.
- tests: test_product_overrides.py; workbook dropdown count -> 14.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013jCVWSz8gVff6mkRLc5LBe
</commit_message>
<xml_diff>
--- a/templates/campaign-plan/Campaign-Plan-Template.xlsx
+++ b/templates/campaign-plan/Campaign-Plan-Template.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:C37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -690,166 +690,274 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>— FORMATS &amp; PRODUCTS —</t>
+          <t>— PRODUCTS (Y/N — blank = brand default; not every campaign runs each) —</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr"/>
-      <c r="C17" s="3" t="inlineStr"/>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Toggle the placements this campaign runs. Blank keeps the brand's standard set.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Formats</t>
+          <t>Include Remnant Video</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>(optional — defaults from Brand) remnant_video | pause_ads | premium_preroll | essential_bumper | cbs_preroll | cbs_after_midroll_bumper | cbs_1z_lockdown | cbs_2z_lockdown | mtve_after_midroll_bumper | bet_after_midroll_bumper</t>
+          <t>(Y/N) — core remnant video; blank = brand default</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Video Domination</t>
+          <t>Include Pause Ads</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>(optional) — pluto | standard | aus_10_streaming | uk_my5</t>
+          <t>(Y/N) — P+ / CBS Network</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>Video Domination Targeting</t>
+          <t>Include Premium Pre-Roll</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>(Pluto VD only) — Pluto categories; semicolon-separated</t>
+          <t>(Y/N) — Paramount+</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Takeover</t>
+          <t>Include Essential Bumper</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>(optional) — hpto | first_impression | arena_takeover | three_peat</t>
+          <t>(Y/N) — Paramount+</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>— OVERRIDES (usually leave blank; auto-derived) —</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr"/>
-      <c r="C22" s="3" t="inlineStr"/>
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Include CBS Pre-Roll</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>(Y/N) — CBS Network</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>Brand</t>
+          <t>Include After Mid-Roll Bumper</t>
         </is>
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>(auto from Campaign) — override only if needed</t>
+          <t>(Y/N) — CBS Network / MTVE / BET</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>Advertiser</t>
+          <t>Include 1Z Lockdown</t>
         </is>
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>(auto from Brand)</t>
+          <t>(Y/N) — CBS Network</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>Advertiser ID</t>
+          <t>Include 2Z Lockdown</t>
         </is>
       </c>
       <c r="B25" t="inlineStr"/>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>(auto)</t>
+          <t>(Y/N) — CBS Network</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>Campaign ID</t>
+          <t>Video Domination</t>
         </is>
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>(auto from Campaign Name)</t>
+          <t>(optional) — pluto | standard | aus_10_streaming | uk_my5</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>Insertion Order Name</t>
+          <t>Video Domination Targeting</t>
         </is>
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>(auto) — defaults to "{Title} - {Region}"</t>
+          <t>(Pluto VD only) — Pluto categories; semicolon-separated</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>Recommended Show</t>
+          <t>Takeover</t>
         </is>
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" s="5" t="inlineStr">
         <is>
+          <t>(optional) — hpto | first_impression | arena_takeover | three_peat</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>— OVERRIDES (usually leave blank; auto-derived) —</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr"/>
+      <c r="C29" s="3" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Formats</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr"/>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>(auto from Brand) override the full set only if the Products toggles aren't enough — remnant_video | pause_ads | premium_preroll | essential_bumper | cbs_preroll | cbs_after_midroll_bumper | cbs_1z_lockdown | cbs_2z_lockdown | mtve_after_midroll_bumper | bet_after_midroll_bumper</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Brand</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr"/>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>(auto from Campaign) — override only if needed</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Advertiser</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr"/>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>(auto from Brand)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Advertiser ID</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr"/>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>(auto)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Campaign ID</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr"/>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>(auto from Campaign Name)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Insertion Order Name</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr"/>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>(auto) — defaults to "{Title} - {Region}"</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Recommended Show</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr"/>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
           <t>(auto) — defaults to Title</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="4" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
         <is>
           <t>Exclude Show</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr"/>
-      <c r="C29" s="5" t="inlineStr">
+      <c r="B37" t="inlineStr"/>
+      <c r="C37" s="5" t="inlineStr">
         <is>
           <t>(auto) — defaults to Title</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="6">
+  <dataValidations count="14">
     <dataValidation sqref="B4" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
       <formula1>_Lists!$A$2:$A$7</formula1>
     </dataValidation>
@@ -859,13 +967,37 @@
     <dataValidation sqref="B10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
       <formula1>_Lists!$C$2:$C$3</formula1>
     </dataValidation>
+    <dataValidation sqref="B18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
+      <formula1>_Lists!$G$2:$G$3</formula1>
+    </dataValidation>
     <dataValidation sqref="B19" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
+      <formula1>_Lists!$G$2:$G$3</formula1>
+    </dataValidation>
+    <dataValidation sqref="B20" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
+      <formula1>_Lists!$G$2:$G$3</formula1>
+    </dataValidation>
+    <dataValidation sqref="B21" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
+      <formula1>_Lists!$G$2:$G$3</formula1>
+    </dataValidation>
+    <dataValidation sqref="B22" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
+      <formula1>_Lists!$G$2:$G$3</formula1>
+    </dataValidation>
+    <dataValidation sqref="B23" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
+      <formula1>_Lists!$G$2:$G$3</formula1>
+    </dataValidation>
+    <dataValidation sqref="B24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
+      <formula1>_Lists!$G$2:$G$3</formula1>
+    </dataValidation>
+    <dataValidation sqref="B25" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
+      <formula1>_Lists!$G$2:$G$3</formula1>
+    </dataValidation>
+    <dataValidation sqref="B26" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
       <formula1>_Lists!$D$2:$D$5</formula1>
     </dataValidation>
-    <dataValidation sqref="B21" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
+    <dataValidation sqref="B28" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
       <formula1>_Lists!$E$2:$E$5</formula1>
     </dataValidation>
-    <dataValidation sqref="B23" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
+    <dataValidation sqref="B31" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
       <formula1>_Lists!$F$2:$F$9</formula1>
     </dataValidation>
   </dataValidations>
@@ -1493,7 +1625,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1527,6 +1659,11 @@
           <t>brand</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>include remnant video</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1559,6 +1696,11 @@
           <t>paramount_plus_domestic</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1589,6 +1731,11 @@
       <c r="F3" t="inlineStr">
         <is>
           <t>cbs_sports</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Pluto En Español brands (simple untargeted remnant)
Model the two Spanish-language remnant brands from their live reference IOs:
- New `pluto_es_remnant` format: flat per-duration lines, no relationship
  targeting, House Pre-Roll on short creatives only (drops at 30s).
- order_builder: flat-line path now honors no_targeting, a brand
  placement_name_suffix, and duration-dependent ad units
  (_ad_units_for_duration).
- brands.yaml: pluto_es_adult (Pluto TV - En Espanol - USA, adv 1000522) and
  pluto_es_kids (Pluto TV - Kids - En Espanol - USA, adv 1000523). The En Español
  Kids brand runs plain remnant (no kids VG targeting), so it is not kids-gated.
- Preview matches the reference IOs exactly (names, ad units per duration, geo
  165, zero targeting sets). tests/test_pluto_es_brands.py. Workbook regenerated.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013jCVWSz8gVff6mkRLc5LBe
</commit_message>
<xml_diff>
--- a/templates/campaign-plan/Campaign-Plan-Template.xlsx
+++ b/templates/campaign-plan/Campaign-Plan-Template.xlsx
@@ -962,7 +962,7 @@
       <formula1>_Lists!$A$2:$A$7</formula1>
     </dataValidation>
     <dataValidation sqref="B5" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
-      <formula1>_Lists!$B$2:$B$9</formula1>
+      <formula1>_Lists!$B$2:$B$11</formula1>
     </dataValidation>
     <dataValidation sqref="B10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
       <formula1>_Lists!$C$2:$C$3</formula1>
@@ -998,7 +998,7 @@
       <formula1>_Lists!$E$2:$E$5</formula1>
     </dataValidation>
     <dataValidation sqref="B31" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
-      <formula1>_Lists!$F$2:$F$9</formula1>
+      <formula1>_Lists!$F$2:$F$11</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1625,7 +1625,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1851,6 +1851,30 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Pluto TV - En Espanol - USA</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>pluto_es_adult</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Pluto TV - Kids - En Espanol - USA</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>pluto_es_kids</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Paramount+ Kids (UK) + reusable format overrides
Build P+ Kids UK from the Kamp Koral reference, adding two small reusable
mechanisms:
- Brand `format_overrides`: per-format template overrides so a region can reuse a
  format (UK bumper "Basic Plan") without a new template.
- Explicit `drop_units` on flat-line ad units: drop only named units at the
  duration threshold (UK P+ line keeps the INTL pre-roll, drops the House
  Pre-Roll at 30s).

P+ Kids UK splits into a P+ line (main [932583], INTL pre-roll) and a Pluto line
(main [1109067,1120870] UK Pluto kids SGs, "(Pluto)" infix), plus Premium
Pre-Roll + Basic Plan Bumper — geo UK (56). New formats pplus_kids_remnant_pplus
/ _pluto; brand paramount_plus_kids_uk. Preview matches the reference exactly.
tests/test_pplus_kids.py; workbook regenerated.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013jCVWSz8gVff6mkRLc5LBe
</commit_message>
<xml_diff>
--- a/templates/campaign-plan/Campaign-Plan-Template.xlsx
+++ b/templates/campaign-plan/Campaign-Plan-Template.xlsx
@@ -962,7 +962,7 @@
       <formula1>_Lists!$A$2:$A$7</formula1>
     </dataValidation>
     <dataValidation sqref="B5" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
-      <formula1>_Lists!$B$2:$B$12</formula1>
+      <formula1>_Lists!$B$2:$B$13</formula1>
     </dataValidation>
     <dataValidation sqref="B10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
       <formula1>_Lists!$C$2:$C$3</formula1>
@@ -998,7 +998,7 @@
       <formula1>_Lists!$E$2:$E$5</formula1>
     </dataValidation>
     <dataValidation sqref="B31" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
-      <formula1>_Lists!$F$2:$F$12</formula1>
+      <formula1>_Lists!$F$2:$F$13</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1625,7 +1625,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1887,6 +1887,18 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Paramount + - Kids - UK</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>paramount_plus_kids_uk</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Pluto TV (UK) — standard tiered remnant, standard genres
UK uses the standard genre VGs (the region-specific VGs in the reference were an
old setup), so Pluto UK mirrors the standard pluto_tv setup: Pluto-only main SG
(929392), the shared genre resolver, region UK (56), Paramount House ad units
(71999/72000/72001). New brand pluto_tv_uk (campaign Pluto TV - UK). Builds the
tiered remnant (Tier 2 Channels / Tier 3 Genre+Categories / Tier 4 RON), no
Tier-1 DDA. tests/test_pluto_uk.py; reference-ios.md updated; workbook regenerated.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013jCVWSz8gVff6mkRLc5LBe
</commit_message>
<xml_diff>
--- a/templates/campaign-plan/Campaign-Plan-Template.xlsx
+++ b/templates/campaign-plan/Campaign-Plan-Template.xlsx
@@ -962,7 +962,7 @@
       <formula1>_Lists!$A$2:$A$7</formula1>
     </dataValidation>
     <dataValidation sqref="B5" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
-      <formula1>_Lists!$B$2:$B$13</formula1>
+      <formula1>_Lists!$B$2:$B$14</formula1>
     </dataValidation>
     <dataValidation sqref="B10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
       <formula1>_Lists!$C$2:$C$3</formula1>
@@ -998,7 +998,7 @@
       <formula1>_Lists!$E$2:$E$5</formula1>
     </dataValidation>
     <dataValidation sqref="B31" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
-      <formula1>_Lists!$F$2:$F$13</formula1>
+      <formula1>_Lists!$F$2:$F$14</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1625,7 +1625,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1899,6 +1899,18 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Pluto TV - UK</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>pluto_tv_uk</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Paramount+ UK (adult): standard tiered model with P+/Pluto split
Add reusable generalizations that make region brands config-driven:
- per-format main_site_groups override (UK P+ line vs Pluto line),
- per-format targeting_kinds routing (P+ line = showlist/genre; Pluto line =
  channels/categories/genre),
- tier_infix ("(Pluto)") appended after the tier in the name,
- duration-dependent ad units on the tiered path too (House Pre-Roll drops at 30s;
  INTL pre-roll stays on P+ lines).
Brand paramount_plus_uk mirrors The Agency: P+ lines + Pluto lines + Pause Ads +
Premium Pre-Roll + Basic Plan Bumper, geo UK. tests/test_pplus_uk.py; 88 passing.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013jCVWSz8gVff6mkRLc5LBe
</commit_message>
<xml_diff>
--- a/templates/campaign-plan/Campaign-Plan-Template.xlsx
+++ b/templates/campaign-plan/Campaign-Plan-Template.xlsx
@@ -962,7 +962,7 @@
       <formula1>_Lists!$A$2:$A$7</formula1>
     </dataValidation>
     <dataValidation sqref="B5" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
-      <formula1>_Lists!$B$2:$B$14</formula1>
+      <formula1>_Lists!$B$2:$B$15</formula1>
     </dataValidation>
     <dataValidation sqref="B10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
       <formula1>_Lists!$C$2:$C$3</formula1>
@@ -998,7 +998,7 @@
       <formula1>_Lists!$E$2:$E$5</formula1>
     </dataValidation>
     <dataValidation sqref="B31" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
-      <formula1>_Lists!$F$2:$F$14</formula1>
+      <formula1>_Lists!$F$2:$F$15</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1625,7 +1625,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1911,6 +1911,18 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Paramount + - UK</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>paramount_plus_uk</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
UK P+ "Include Pluto" checkbox + region has_pluto flags (AU/IE no Pluto)
- UK P+ Pluto breakout lines are now OFF by default and opt-in via an "Include
  Pluto" checkbox (product toggle pluto_breakout -> pplus_uk_remnant_pluto in the
  brand's optional_formats). Off = P+ lines + pause + guaranteed (11); on = adds
  the 6 Pluto breakout lines (17).
- regions.yaml: has_pluto flag (default true); AU and new IE (Ireland, country 73)
  = false — no Pluto — for the combined-region builds to come.
- Template Products row + Salesforce Include_Pluto__c + workbook dropdown; test
  count derives from the toggle list.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013jCVWSz8gVff6mkRLc5LBe
</commit_message>
<xml_diff>
--- a/templates/campaign-plan/Campaign-Plan-Template.xlsx
+++ b/templates/campaign-plan/Campaign-Plan-Template.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -807,146 +807,146 @@
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>Video Domination</t>
+          <t>Include Pluto</t>
         </is>
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>(optional) — pluto | standard | aus_10_streaming | uk_my5</t>
+          <t>(Y/N) — UK Paramount+ only; adds the Pluto breakout lines</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>Video Domination Targeting</t>
+          <t>Video Domination</t>
         </is>
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>(Pluto VD only) — Pluto categories; semicolon-separated</t>
+          <t>(optional) — pluto | standard | aus_10_streaming | uk_my5</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>Takeover</t>
+          <t>Video Domination Targeting</t>
         </is>
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" s="5" t="inlineStr">
         <is>
+          <t>(Pluto VD only) — Pluto categories; semicolon-separated</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Takeover</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr"/>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
           <t>(optional) — hpto | first_impression | arena_takeover | three_peat</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>— OVERRIDES (usually leave blank; auto-derived) —</t>
         </is>
       </c>
-      <c r="B29" s="2" t="inlineStr"/>
-      <c r="C29" s="3" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>Formats</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr"/>
-      <c r="C30" s="5" t="inlineStr">
-        <is>
-          <t>(auto from Brand) override the full set only if the Products toggles aren't enough — remnant_video | pause_ads | premium_preroll | essential_bumper | cbs_preroll | cbs_after_midroll_bumper | cbs_1z_lockdown | cbs_2z_lockdown | mtve_after_midroll_bumper | bet_after_midroll_bumper</t>
-        </is>
-      </c>
+      <c r="B30" s="2" t="inlineStr"/>
+      <c r="C30" s="3" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>Brand</t>
+          <t>Formats</t>
         </is>
       </c>
       <c r="B31" t="inlineStr"/>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>(auto from Campaign) — override only if needed</t>
+          <t>(auto from Brand) override the full set only if the Products toggles aren't enough — remnant_video | pause_ads | premium_preroll | essential_bumper | cbs_preroll | cbs_after_midroll_bumper | cbs_1z_lockdown | cbs_2z_lockdown | mtve_after_midroll_bumper | bet_after_midroll_bumper</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>Advertiser</t>
+          <t>Brand</t>
         </is>
       </c>
       <c r="B32" t="inlineStr"/>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>(auto from Brand)</t>
+          <t>(auto from Campaign) — override only if needed</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>Advertiser ID</t>
+          <t>Advertiser</t>
         </is>
       </c>
       <c r="B33" t="inlineStr"/>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>(auto)</t>
+          <t>(auto from Brand)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>Campaign ID</t>
+          <t>Advertiser ID</t>
         </is>
       </c>
       <c r="B34" t="inlineStr"/>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>(auto from Campaign Name)</t>
+          <t>(auto)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>Insertion Order Name</t>
+          <t>Campaign ID</t>
         </is>
       </c>
       <c r="B35" t="inlineStr"/>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>(auto) — defaults to "{Title} - {Region}"</t>
+          <t>(auto from Campaign Name)</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>Recommended Show</t>
+          <t>Insertion Order Name</t>
         </is>
       </c>
       <c r="B36" t="inlineStr"/>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>(auto) — defaults to Title</t>
+          <t>(auto) — defaults to "{Title} - {Region}"</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>Exclude Show</t>
+          <t>Recommended Show</t>
         </is>
       </c>
       <c r="B37" t="inlineStr"/>
@@ -956,10 +956,23 @@
         </is>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Exclude Show</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr"/>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>(auto) — defaults to Title</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <dataValidations count="14">
+  <dataValidations count="15">
     <dataValidation sqref="B4" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
-      <formula1>_Lists!$A$2:$A$7</formula1>
+      <formula1>_Lists!$A$2:$A$8</formula1>
     </dataValidation>
     <dataValidation sqref="B5" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
       <formula1>_Lists!$B$2:$B$15</formula1>
@@ -992,12 +1005,15 @@
       <formula1>_Lists!$G$2:$G$3</formula1>
     </dataValidation>
     <dataValidation sqref="B26" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
+      <formula1>_Lists!$G$2:$G$3</formula1>
+    </dataValidation>
+    <dataValidation sqref="B27" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
       <formula1>_Lists!$D$2:$D$5</formula1>
     </dataValidation>
-    <dataValidation sqref="B28" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
+    <dataValidation sqref="B29" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
       <formula1>_Lists!$E$2:$E$5</formula1>
     </dataValidation>
-    <dataValidation sqref="B31" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
+    <dataValidation sqref="B32" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
       <formula1>_Lists!$F$2:$F$15</formula1>
     </dataValidation>
   </dataValidations>
@@ -1828,6 +1844,11 @@
       </c>
     </row>
     <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>IE</t>
+        </is>
+      </c>
       <c r="B8" t="inlineStr">
         <is>
           <t>Pluto TV - USA</t>

</xml_diff>

<commit_message>
Finish CA brands: Pluto French/Kids, Nick + language field
- pluto_ca_kids_en, nick_ca_en: kids brands, Pluto-only (929392), not tiered,
  age-driven VGs (Nick uses "(Pluto)" infix) — via pplus_kids_remnant +
  format_overrides.
- pluto_ca_fr: plain remnant, no targeting ("Sur Pluto TV" / French - CA).
- No active French P+ CA (English P+ adult + kids only).
- Add `language` field (English/French) to the model, Plan tab, and Salesforce
  (Language__c) for multi-language region routing. 97 passing.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013jCVWSz8gVff6mkRLc5LBe
</commit_message>
<xml_diff>
--- a/templates/campaign-plan/Campaign-Plan-Template.xlsx
+++ b/templates/campaign-plan/Campaign-Plan-Template.xlsx
@@ -975,7 +975,7 @@
       <formula1>_Lists!$A$2:$A$8</formula1>
     </dataValidation>
     <dataValidation sqref="B5" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
-      <formula1>_Lists!$B$2:$B$15</formula1>
+      <formula1>_Lists!$B$2:$B$21</formula1>
     </dataValidation>
     <dataValidation sqref="B10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
       <formula1>_Lists!$C$2:$C$3</formula1>
@@ -1014,7 +1014,7 @@
       <formula1>_Lists!$E$2:$E$5</formula1>
     </dataValidation>
     <dataValidation sqref="B32" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
-      <formula1>_Lists!$F$2:$F$15</formula1>
+      <formula1>_Lists!$F$2:$F$21</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1641,7 +1641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1944,6 +1944,78 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Pluto TV - English - CA</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>pluto_ca_en</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Paramount + - English - CA</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>paramount_plus_ca</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Paramount + - Kids - English - CA</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>paramount_plus_kids_ca</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Pluto TV - Kids - English - CA</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>pluto_ca_kids_en</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Nick - Kids - English - CA</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>nick_ca_en</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Pluto TV - French - CA</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>pluto_ca_fr</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
AU: add Network 10 (10 Streaming) opt-in + rating-restrictions form option
Network 10 (AU) as an "Include Network 10" toggle: adds tiered (10 Streaming)
remnant lines (Net10 Live pre-roll + Paramount House units, Ten Play/CBS Local/
VCBS main SGs, "(10 Streaming)" tier infix, pre-roll drops at 30s). Off by
default; opt in via the Products toggle / Include_Network_10__c.

Rating restrictions: new per-campaign plan.rating_restrictions field (VG values
Network 10 sometimes supplies). Applied as set-level excludes only on formats
flagged applies_rating_restrictions (the 10 Streaming lines) — never on the
standard P+ AU lines. Wired through the plan template, gsheets and Salesforce
Case field map.

Adds test_network_10 (gating, naming/geo, main SGs/ad units, rating-restriction
scoping). Full suite: 106 passing.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013jCVWSz8gVff6mkRLc5LBe
</commit_message>
<xml_diff>
--- a/templates/campaign-plan/Campaign-Plan-Template.xlsx
+++ b/templates/campaign-plan/Campaign-Plan-Template.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C38"/>
+  <dimension ref="A1:C40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -820,162 +820,188 @@
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>Video Domination</t>
+          <t>Include Network 10</t>
         </is>
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>(optional) — pluto | standard | aus_10_streaming | uk_my5</t>
+          <t>(Y/N) — AU Paramount+ only; adds the (10 Streaming) tiered lines</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>Video Domination Targeting</t>
+          <t>Rating Restrictions</t>
         </is>
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>(Pluto VD only) — Pluto categories; semicolon-separated</t>
+          <t>(AU Network 10 only) — VG rating restrictions to exclude; semicolon-separated</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>Takeover</t>
+          <t>Video Domination</t>
         </is>
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>(optional) — hpto | first_impression | arena_takeover | three_peat</t>
+          <t>(optional) — pluto | standard | aus_10_streaming | uk_my5</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>— OVERRIDES (usually leave blank; auto-derived) —</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr"/>
-      <c r="C30" s="3" t="inlineStr"/>
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Video Domination Targeting</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr"/>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>(Pluto VD only) — Pluto categories; semicolon-separated</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>Formats</t>
+          <t>Takeover</t>
         </is>
       </c>
       <c r="B31" t="inlineStr"/>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>(auto from Brand) override the full set only if the Products toggles aren't enough — remnant_video | pause_ads | premium_preroll | essential_bumper | cbs_preroll | cbs_after_midroll_bumper | cbs_1z_lockdown | cbs_2z_lockdown | mtve_after_midroll_bumper | bet_after_midroll_bumper</t>
+          <t>(optional) — hpto | first_impression | arena_takeover | three_peat</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>Brand</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr"/>
-      <c r="C32" s="5" t="inlineStr">
-        <is>
-          <t>(auto from Campaign) — override only if needed</t>
-        </is>
-      </c>
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>— OVERRIDES (usually leave blank; auto-derived) —</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr"/>
+      <c r="C32" s="3" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>Advertiser</t>
+          <t>Formats</t>
         </is>
       </c>
       <c r="B33" t="inlineStr"/>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>(auto from Brand)</t>
+          <t>(auto from Brand) override the full set only if the Products toggles aren't enough — remnant_video | pause_ads | premium_preroll | essential_bumper | cbs_preroll | cbs_after_midroll_bumper | cbs_1z_lockdown | cbs_2z_lockdown | mtve_after_midroll_bumper | bet_after_midroll_bumper</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>Advertiser ID</t>
+          <t>Brand</t>
         </is>
       </c>
       <c r="B34" t="inlineStr"/>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>(auto)</t>
+          <t>(auto from Campaign) — override only if needed</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>Campaign ID</t>
+          <t>Advertiser</t>
         </is>
       </c>
       <c r="B35" t="inlineStr"/>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>(auto from Campaign Name)</t>
+          <t>(auto from Brand)</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>Insertion Order Name</t>
+          <t>Advertiser ID</t>
         </is>
       </c>
       <c r="B36" t="inlineStr"/>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>(auto) — defaults to "{Title} - {Region}"</t>
+          <t>(auto)</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>Recommended Show</t>
+          <t>Campaign ID</t>
         </is>
       </c>
       <c r="B37" t="inlineStr"/>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>(auto) — defaults to Title</t>
+          <t>(auto from Campaign Name)</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>Exclude Show</t>
+          <t>Insertion Order Name</t>
         </is>
       </c>
       <c r="B38" t="inlineStr"/>
       <c r="C38" s="5" t="inlineStr">
         <is>
+          <t>(auto) — defaults to "{Title} - {Region}"</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Recommended Show</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr"/>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
           <t>(auto) — defaults to Title</t>
         </is>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Exclude Show</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr"/>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>(auto) — defaults to Title</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <dataValidations count="15">
+  <dataValidations count="16">
     <dataValidation sqref="B4" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
       <formula1>_Lists!$A$2:$A$8</formula1>
     </dataValidation>
     <dataValidation sqref="B5" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
-      <formula1>_Lists!$B$2:$B$21</formula1>
+      <formula1>_Lists!$B$2:$B$22</formula1>
     </dataValidation>
     <dataValidation sqref="B10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
       <formula1>_Lists!$C$2:$C$3</formula1>
@@ -1008,13 +1034,16 @@
       <formula1>_Lists!$G$2:$G$3</formula1>
     </dataValidation>
     <dataValidation sqref="B27" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
+      <formula1>_Lists!$G$2:$G$3</formula1>
+    </dataValidation>
+    <dataValidation sqref="B29" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
       <formula1>_Lists!$D$2:$D$5</formula1>
     </dataValidation>
-    <dataValidation sqref="B29" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
+    <dataValidation sqref="B31" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
       <formula1>_Lists!$E$2:$E$5</formula1>
     </dataValidation>
-    <dataValidation sqref="B32" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
-      <formula1>_Lists!$F$2:$F$21</formula1>
+    <dataValidation sqref="B34" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
+      <formula1>_Lists!$F$2:$F$22</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1641,7 +1670,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2016,6 +2045,18 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Paramount + - AU</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>paramount_plus_au</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Templates: align the plan/targeting sheets with the field map
- Plan sheet: add Language (CA routing) + fix the stale Region hint (all 15 regions).
- Targeting sheet: add the Kids Audience column (older/younger — Kids brands).
- Workbook builder: add a Language (English/French) dropdown; regenerate
  Campaign-Plan-Template.xlsx. Both sheets now match CASE_FIELD_MAP / the parser.

Updates the workbook dropdown-count test. Full suite: 163 passing.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013jCVWSz8gVff6mkRLc5LBe
</commit_message>
<xml_diff>
--- a/templates/campaign-plan/Campaign-Plan-Template.xlsx
+++ b/templates/campaign-plan/Campaign-Plan-Template.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C40"/>
+  <dimension ref="A1:C41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -515,152 +515,152 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>(required) — USA | CA | AU | LATAM | BR | UK</t>
+          <t>(required) — USA | CA | UK | IE | AU | LATAM | BR | FR | IT | GSA | FI | DK | NO | SE | ES</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Campaign Name</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Paramount + - USA</t>
-        </is>
-      </c>
+          <t>Language</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>(required) — Paramount + - USA | CBS Sports - USA | CBS News - USA | CBS Network - USA | MTVE - USA | BET Media Group - USA | Pluto TV - USA | Pluto TV (Cross-Company) - USA</t>
+          <t>(CA only) — English | French; routes to the FR vs EN advertiser</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
+          <t>Campaign Name</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Paramount + - USA</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>(required) — Paramount + - USA | CBS Sports - USA | CBS News - USA | CBS Network - USA | MTVE - USA | BET Media Group - USA | Pluto TV - USA | Pluto TV (Cross-Company) - USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
           <t>Salesforce Case</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>(auto — from the Case)</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>— CREATIVE / NAMING —</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr"/>
-      <c r="C7" s="3" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Season or Messaging</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Season 1</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>(optional) — middle of the placement name</t>
-        </is>
-      </c>
+      <c r="B8" s="2" t="inlineStr"/>
+      <c r="C8" s="3" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Video Durations</t>
+          <t>Season or Messaging</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>30; 15</t>
+          <t>Season 1</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>(required for video) — seconds; semicolon-separated</t>
+          <t>(optional) — middle of the placement name</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Content Type</t>
+          <t>Video Durations</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>show</t>
+          <t>30; 15</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>show | movie</t>
+          <t>(required for video) — seconds; semicolon-separated</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Content ID</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr"/>
+          <t>Content Type</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>show</t>
+        </is>
+      </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>(CM) — ShowID/MovieID; fills [ShowID:] + Recommended Show</t>
+          <t>show | movie</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Recommended Show ID</t>
+          <t>Content ID</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" s="5" t="inlineStr">
         <is>
+          <t>(CM) — ShowID/MovieID; fills [ShowID:] + Recommended Show</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Recommended Show ID</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
           <t>(CM) — defaults to Content ID</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>— FLIGHTING —</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr"/>
-      <c r="C13" s="3" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>Flight Start</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>(required) — YYYY-MM-DD</t>
-        </is>
-      </c>
+      <c r="B14" s="2" t="inlineStr"/>
+      <c r="C14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Flight End</t>
+          <t>Flight Start</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
@@ -673,76 +673,76 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
+          <t>Flight End</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>(required) — YYYY-MM-DD</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
           <t>Flight Code</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>L1</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="C17" s="5" t="inlineStr">
         <is>
           <t>(optional)</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>— PRODUCTS (Y/N — blank = brand default; not every campaign runs each) —</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr"/>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr"/>
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>Toggle the placements this campaign runs. Blank keeps the brand's standard set.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>Include Remnant Video</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>(Y/N) — core remnant video; blank = brand default</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Include Pause Ads</t>
+          <t>Include Remnant Video</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>(Y/N) — P+ / CBS Network</t>
+          <t>(Y/N) — core remnant video; blank = brand default</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>Include Premium Pre-Roll</t>
+          <t>Include Pause Ads</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>(Y/N) — Paramount+</t>
+          <t>(Y/N) — P+ / CBS Network</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Include Essential Bumper</t>
+          <t>Include Premium Pre-Roll</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
@@ -755,46 +755,46 @@
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>Include CBS Pre-Roll</t>
+          <t>Include Essential Bumper</t>
         </is>
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>(Y/N) — CBS Network</t>
+          <t>(Y/N) — Paramount+</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>Include After Mid-Roll Bumper</t>
+          <t>Include CBS Pre-Roll</t>
         </is>
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>(Y/N) — CBS Network / MTVE / BET</t>
+          <t>(Y/N) — CBS Network</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>Include 1Z Lockdown</t>
+          <t>Include After Mid-Roll Bumper</t>
         </is>
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>(Y/N) — CBS Network</t>
+          <t>(Y/N) — CBS Network / MTVE / BET</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>Include 2Z Lockdown</t>
+          <t>Include 1Z Lockdown</t>
         </is>
       </c>
       <c r="B25" t="inlineStr"/>
@@ -807,185 +807,185 @@
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>Include Pluto</t>
+          <t>Include 2Z Lockdown</t>
         </is>
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>(Y/N) — UK Paramount+ only; adds the Pluto breakout lines</t>
+          <t>(Y/N) — CBS Network</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>Include Network 10</t>
+          <t>Include Pluto</t>
         </is>
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>(Y/N) — AU Paramount+ only; adds the (10 Streaming) tiered lines</t>
+          <t>(Y/N) — UK Paramount+ only; adds the Pluto breakout lines</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>Rating Restrictions</t>
+          <t>Include Network 10</t>
         </is>
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>(AU Network 10 only) — VG rating restrictions to exclude; semicolon-separated</t>
+          <t>(Y/N) — AU Paramount+ only; adds the (10 Streaming) tiered lines</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>Video Domination</t>
+          <t>Rating Restrictions</t>
         </is>
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>(optional) — pluto | standard | aus_10_streaming | uk_my5</t>
+          <t>(AU Network 10 only) — VG rating restrictions to exclude; semicolon-separated</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>Video Domination Targeting</t>
+          <t>Video Domination</t>
         </is>
       </c>
       <c r="B30" t="inlineStr"/>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>(Pluto VD only) — Pluto categories; semicolon-separated</t>
+          <t>(optional) — pluto | standard | aus_10_streaming | uk_my5</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>Takeover</t>
+          <t>Video Domination Targeting</t>
         </is>
       </c>
       <c r="B31" t="inlineStr"/>
       <c r="C31" s="5" t="inlineStr">
         <is>
+          <t>(Pluto VD only) — Pluto categories; semicolon-separated</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Takeover</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr"/>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
           <t>(optional) — hpto | first_impression | arena_takeover | three_peat</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
         <is>
           <t>— OVERRIDES (usually leave blank; auto-derived) —</t>
         </is>
       </c>
-      <c r="B32" s="2" t="inlineStr"/>
-      <c r="C32" s="3" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="4" t="inlineStr">
-        <is>
-          <t>Formats</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr"/>
-      <c r="C33" s="5" t="inlineStr">
-        <is>
-          <t>(auto from Brand) override the full set only if the Products toggles aren't enough — remnant_video | pause_ads | premium_preroll | essential_bumper | cbs_preroll | cbs_after_midroll_bumper | cbs_1z_lockdown | cbs_2z_lockdown | mtve_after_midroll_bumper | bet_after_midroll_bumper</t>
-        </is>
-      </c>
+      <c r="B33" s="2" t="inlineStr"/>
+      <c r="C33" s="3" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>Brand</t>
+          <t>Formats</t>
         </is>
       </c>
       <c r="B34" t="inlineStr"/>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>(auto from Campaign) — override only if needed</t>
+          <t>(auto from Brand) override the full set only if the Products toggles aren't enough — remnant_video | pause_ads | premium_preroll | essential_bumper | cbs_preroll | cbs_after_midroll_bumper | cbs_1z_lockdown | cbs_2z_lockdown | mtve_after_midroll_bumper | bet_after_midroll_bumper</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>Advertiser</t>
+          <t>Brand</t>
         </is>
       </c>
       <c r="B35" t="inlineStr"/>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>(auto from Brand)</t>
+          <t>(auto from Campaign) — override only if needed</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>Advertiser ID</t>
+          <t>Advertiser</t>
         </is>
       </c>
       <c r="B36" t="inlineStr"/>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>(auto)</t>
+          <t>(auto from Brand)</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>Campaign ID</t>
+          <t>Advertiser ID</t>
         </is>
       </c>
       <c r="B37" t="inlineStr"/>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>(auto from Campaign Name)</t>
+          <t>(auto)</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>Insertion Order Name</t>
+          <t>Campaign ID</t>
         </is>
       </c>
       <c r="B38" t="inlineStr"/>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>(auto) — defaults to "{Title} - {Region}"</t>
+          <t>(auto from Campaign Name)</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>Recommended Show</t>
+          <t>Insertion Order Name</t>
         </is>
       </c>
       <c r="B39" t="inlineStr"/>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>(auto) — defaults to Title</t>
+          <t>(auto) — defaults to "{Title} - {Region}"</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>Exclude Show</t>
+          <t>Recommended Show</t>
         </is>
       </c>
       <c r="B40" t="inlineStr"/>
@@ -995,55 +995,71 @@
         </is>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Exclude Show</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr"/>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>(auto) — defaults to Title</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <dataValidations count="16">
+  <dataValidations count="17">
     <dataValidation sqref="B4" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
-      <formula1>_Lists!$A$2:$A$8</formula1>
+      <formula1>_Lists!$A$2:$A$16</formula1>
     </dataValidation>
     <dataValidation sqref="B5" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
-      <formula1>_Lists!$B$2:$B$22</formula1>
+      <formula1>_Lists!$B$2:$B$3</formula1>
     </dataValidation>
-    <dataValidation sqref="B10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
-      <formula1>_Lists!$C$2:$C$3</formula1>
+    <dataValidation sqref="B6" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
+      <formula1>_Lists!$C$2:$C$80</formula1>
     </dataValidation>
-    <dataValidation sqref="B18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
-      <formula1>_Lists!$G$2:$G$3</formula1>
+    <dataValidation sqref="B11" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
+      <formula1>_Lists!$D$2:$D$3</formula1>
     </dataValidation>
     <dataValidation sqref="B19" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
-      <formula1>_Lists!$G$2:$G$3</formula1>
+      <formula1>_Lists!$H$2:$H$3</formula1>
     </dataValidation>
     <dataValidation sqref="B20" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
-      <formula1>_Lists!$G$2:$G$3</formula1>
+      <formula1>_Lists!$H$2:$H$3</formula1>
     </dataValidation>
     <dataValidation sqref="B21" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
-      <formula1>_Lists!$G$2:$G$3</formula1>
+      <formula1>_Lists!$H$2:$H$3</formula1>
     </dataValidation>
     <dataValidation sqref="B22" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
-      <formula1>_Lists!$G$2:$G$3</formula1>
+      <formula1>_Lists!$H$2:$H$3</formula1>
     </dataValidation>
     <dataValidation sqref="B23" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
-      <formula1>_Lists!$G$2:$G$3</formula1>
+      <formula1>_Lists!$H$2:$H$3</formula1>
     </dataValidation>
     <dataValidation sqref="B24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
-      <formula1>_Lists!$G$2:$G$3</formula1>
+      <formula1>_Lists!$H$2:$H$3</formula1>
     </dataValidation>
     <dataValidation sqref="B25" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
-      <formula1>_Lists!$G$2:$G$3</formula1>
+      <formula1>_Lists!$H$2:$H$3</formula1>
     </dataValidation>
     <dataValidation sqref="B26" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
-      <formula1>_Lists!$G$2:$G$3</formula1>
+      <formula1>_Lists!$H$2:$H$3</formula1>
     </dataValidation>
     <dataValidation sqref="B27" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
-      <formula1>_Lists!$G$2:$G$3</formula1>
+      <formula1>_Lists!$H$2:$H$3</formula1>
     </dataValidation>
-    <dataValidation sqref="B29" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
-      <formula1>_Lists!$D$2:$D$5</formula1>
+    <dataValidation sqref="B28" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
+      <formula1>_Lists!$H$2:$H$3</formula1>
     </dataValidation>
-    <dataValidation sqref="B31" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
+    <dataValidation sqref="B30" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
       <formula1>_Lists!$E$2:$E$5</formula1>
     </dataValidation>
-    <dataValidation sqref="B34" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
-      <formula1>_Lists!$F$2:$F$22</formula1>
+    <dataValidation sqref="B32" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
+      <formula1>_Lists!$F$2:$F$5</formula1>
+    </dataValidation>
+    <dataValidation sqref="B35" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Pick a value from the list." prompt="Choose from the dropdown." type="list">
+      <formula1>_Lists!$G$2:$G$80</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1056,7 +1072,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:G35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1065,6 +1081,7 @@
     <col width="24" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1096,6 +1113,11 @@
       <c r="F1" s="6" t="inlineStr">
         <is>
           <t>Pluto Channels</t>
+        </is>
+      </c>
+      <c r="G1" s="6" t="inlineStr">
+        <is>
+          <t>Kids Audience (older / younger — Kids brands only)</t>
         </is>
       </c>
     </row>
@@ -1670,7 +1692,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:H80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1681,30 +1703,35 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>language</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>campaign name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>content type</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>video domination</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>takeover</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>brand</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>include remnant video</t>
         </is>
@@ -1718,30 +1745,35 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>Paramount + - USA</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>show</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>pluto</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>hpto</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>paramount_plus_domestic</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -1755,30 +1787,35 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>French</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>CBS Sports - USA</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>movie</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>standard</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>first_impression</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>cbs_sports</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1790,22 +1827,22 @@
           <t>AU</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>CBS News - USA</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>aus_10_streaming</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>arena_takeover</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>cbs_news</t>
         </is>
@@ -1817,22 +1854,22 @@
           <t>LATAM</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>CBS Network - USA</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>uk_my5</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>three_peat</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>cbs_network</t>
         </is>
@@ -1844,12 +1881,12 @@
           <t>BR</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>MTVE - USA</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>mtve</t>
         </is>
@@ -1861,12 +1898,12 @@
           <t>UK</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>BET Media Group - USA</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>bet</t>
         </is>
@@ -1878,182 +1915,918 @@
           <t>IE</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>Pluto TV - USA</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>pluto_tv</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="B9" t="inlineStr">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
         <is>
           <t>Pluto TV (Cross-Company) - USA</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>pluto_tv_xco</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="B10" t="inlineStr">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
         <is>
           <t>Pluto TV - En Espanol - USA</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>pluto_es_adult</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="B11" t="inlineStr">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>GSA</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
         <is>
           <t>Pluto TV - Kids - En Espanol - USA</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>pluto_es_kids</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="B12" t="inlineStr">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>FI</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
         <is>
           <t>Paramount + - Kids - USA</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>paramount_plus_kids</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="B13" t="inlineStr">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>DK</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
         <is>
           <t>Paramount + - Kids - UK</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>paramount_plus_kids_uk</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="B14" t="inlineStr">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
         <is>
           <t>Pluto TV - UK</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>pluto_tv_uk</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="B15" t="inlineStr">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>SE</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
         <is>
           <t>Paramount + - UK</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>paramount_plus_uk</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="B16" t="inlineStr">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Paramount + - IE</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>paramount_plus_ie</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Paramount + - Kids - IE</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>paramount_plus_kids_ie</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Paramount + - LATAM</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>paramount_plus_latam</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Pluto TV - LATAM</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>pluto_tv_latam</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Paramount + - Kids - LATAM</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>paramount_plus_kids_latam</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Nick - Kids - LATAM</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>nick_latam</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Nick Jr. - Kids - LATAM</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>nick_jr_latam</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="C23" t="inlineStr">
         <is>
           <t>Pluto TV - English - CA</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="G23" t="inlineStr">
         <is>
           <t>pluto_ca_en</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="B17" t="inlineStr">
+    <row r="24">
+      <c r="C24" t="inlineStr">
         <is>
           <t>Paramount + - English - CA</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="G24" t="inlineStr">
         <is>
           <t>paramount_plus_ca</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="B18" t="inlineStr">
+    <row r="25">
+      <c r="C25" t="inlineStr">
         <is>
           <t>Paramount + - Kids - English - CA</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="G25" t="inlineStr">
         <is>
           <t>paramount_plus_kids_ca</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="B19" t="inlineStr">
+    <row r="26">
+      <c r="C26" t="inlineStr">
         <is>
           <t>Pluto TV - Kids - English - CA</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="G26" t="inlineStr">
         <is>
           <t>pluto_ca_kids_en</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="B20" t="inlineStr">
+    <row r="27">
+      <c r="C27" t="inlineStr">
         <is>
           <t>Nick - Kids - English - CA</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="G27" t="inlineStr">
         <is>
           <t>nick_ca_en</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="B21" t="inlineStr">
+    <row r="28">
+      <c r="C28" t="inlineStr">
         <is>
           <t>Pluto TV - French - CA</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="G28" t="inlineStr">
         <is>
           <t>pluto_ca_fr</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="B22" t="inlineStr">
+    <row r="29">
+      <c r="C29" t="inlineStr">
         <is>
           <t>Paramount + - AU</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="G29" t="inlineStr">
         <is>
           <t>paramount_plus_au</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Nick - Kids - AU</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>nick_au</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Nick Jr. - Kids - AU</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>nick_jr_au</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Paramount + - BR</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>paramount_plus_br</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Pluto TV - BR</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>pluto_tv_br</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Paramount + - Kids - BR</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>paramount_plus_kids_br</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Nick - Kids - BR</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>nick_br</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Nick Jr - Kids - BR</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>nick_jr_br</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Paramount + - FR</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>paramount_plus_fr</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Paramount + - Kids - FR</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>paramount_plus_kids_fr</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Pluto TV - FR</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>pluto_tv_fr</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Pluto TV - Kids - FR</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>pluto_tv_kids_fr</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Nick - Kids - FR</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>nick_fr</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Paramount + - IT</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>paramount_plus_it</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Paramount + - Kids  - IT</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>paramount_plus_kids_it</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Pluto TV - IT</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>pluto_tv_it</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Pluto TV - Kids - IT</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>pluto_tv_kids_it</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Nickelodeon - Kids - IT</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>nick_it</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Paramount + - GSA</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>paramount_plus_gsa</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Paramount + - Kids - GSA</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>paramount_plus_kids_gsa</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Pluto TV - GSA</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>pluto_tv_gsa</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Pluto TV - Kids - GSA</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>pluto_tv_kids_gsa</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Nick - Kids - GSA</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>nick_gsa</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Pluto TV - FI</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>pluto_tv_fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Pluto TV - Kids - FI</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>pluto_tv_kids_fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Nick - Kids - FI</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>nick_fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Pluto TV - DK</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>pluto_tv_dk</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Pluto TV - Kids - DK</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>pluto_tv_kids_dk</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Nick - Kids - DK</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>nick_dk</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Pluto TV - NO</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>pluto_tv_no</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Pluto TV - Kids - NO</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>pluto_tv_kids_no</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Nick - Kids - NO</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>nick_no</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Pluto TV - SE</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>pluto_tv_se</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Pluto TV - Kids - SE</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>pluto_tv_kids_se</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Nick - Kids - SE</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>nick_se</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Pluto TV - ES</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>pluto_tv_es</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Pluto TV - Kids - ES</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>pluto_tv_kids_es</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Nick - Kids - ES</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>nick_es</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Nick Jr. - Kids - ES</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>nick_jr_es</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Paramount Pictures - UK</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>paramount_pictures_uk</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Paramount Pictures - FR</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>paramount_pictures_fr</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Paramount Pictures - IT</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>paramount_pictures_it</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Paramount Pictures - GSA</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>paramount_pictures_gsa</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Paramount Pictures - DK</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>paramount_pictures_dk</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Paramount Pictures - FI</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>paramount_pictures_fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Paramount Pictures - NO</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>paramount_pictures_no</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Paramount Pictures - SE</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>paramount_pictures_se</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Paramount Pictures - ES</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>paramount_pictures_es</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Paramount Pictures - LATAM</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>paramount_pictures_latam</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Paramount Pictures - BR</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>paramount_pictures_br</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Paramount Pictures - Kids - BR</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>paramount_pictures_kids_br</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Paramount Consumer Products - Kids - BR</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>paramount_consumer_products_kids_br</t>
         </is>
       </c>
     </row>

</xml_diff>